<commit_message>
Google Sheet sin NA, preguntas cubren todos los datasets, nota final por entregas y portada local
Republicación desde el curso privado: ver detalle en el commit 3bee4cc de
AEDV_2026_2027.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RubricaEvaluaciónProyectoPersonal.xlsx
+++ b/RubricaEvaluaciónProyectoPersonal.xlsx
@@ -1,22 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1536" yWindow="1536" windowWidth="14316" windowHeight="13332" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="14316" windowHeight="13332" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t xml:space="preserve">Preguntas de investigación: se plantean preguntas de investigación interesantes, concretas y que se pueden responder con los datos, que justifican la elección de los datasets y cubren todos los datasets elegidos (no puede haber datasets sin una pregunta que los justifique). La estrategia de selección y el uso de la IA se describen en Comprensión del negocio. Las preguntas iniciales se van refinando por iteraciones a partir del análisis de los datos y se responden en las conclusiones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uso Google Sheet para el control dedicación proyecto: la hoja está operativa desde el principio y no tiene actividades incompletas (sin fecha de inicio, sin fecha de fin o sin minutos calculados) ni valores NA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega memoria en html y código en Rmd que solo use librerías usadas en la asignatura, con ficheros de datos en formato RDS. El código debe incluir todo lo necesario para compilar localmente en cualquier ordenador, incluida la imagen de portada como fichero local (no un enlace externo).</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,25 +38,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
+      <b/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FF1F4E79"/>
-      <sz val="10"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF1F4E79"/>
       <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="6">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -82,30 +101,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -462,16 +482,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="84.5546875" customWidth="1" min="2" max="2"/>
+    <col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="84.5546875" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.95" customHeight="1">
@@ -487,7 +507,7 @@
       </c>
     </row>
     <row r="2" ht="16.05" customHeight="1">
-      <c r="A2" s="2" t="n"/>
+      <c r="A2" s="2"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Alcance y calidad global</t>
@@ -512,14 +532,12 @@
           <t>1,2,3</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Preguntas de investigación: se plantean preguntas de investigación interesantes, concretas y que se pueden responder con los datos, que justifican la elección de los datasets (la estrategia de selección y el uso de la IA se describen en Comprensión del negocio). Las preguntas iniciales se van refinando por iteraciones a partir del análisis de los datos y se responden en las conclusiones.</t>
-        </is>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="5" ht="40.2" customHeight="1">
-      <c r="A5" s="2" t="n"/>
+      <c r="A5" s="2"/>
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Entrega y formato técnico</t>
@@ -532,10 +550,8 @@
           <t>1,2,3</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Entrega memoria en html y código en Rmd que solo use librerías usadas en la asignatura, con ficheros de datos en formato RDS. El código debe incluir todo lo necesario para compilar localmente en cualquier ordenador.</t>
-        </is>
+      <c r="B6" s="7" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="7" ht="31.95" customHeight="1">
@@ -563,7 +579,7 @@
       </c>
     </row>
     <row r="9" ht="31.95" customHeight="1">
-      <c r="A9" s="2" t="n"/>
+      <c r="A9" s="2"/>
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Texto y estructura de la memoria</t>
@@ -602,7 +618,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Todas las secciones están completadas correctamente siguiendo la metodología CRISP-DM </t>
+          <t>xml:space="preserve"&gt; Todas las secciones están completadas correctamente siguiendo la metodología CRISP-DM </t>
         </is>
       </c>
     </row>
@@ -631,7 +647,7 @@
       </c>
     </row>
     <row r="15" ht="31.95" customHeight="1">
-      <c r="A15" s="2" t="n"/>
+      <c r="A15" s="2"/>
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Comprensión y preparación de los datos</t>
@@ -646,7 +662,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incluye correctamente la información/origen/fiabilidad de los datasets </t>
+          <t>xml:space="preserve"&gt;Incluye correctamente la información/origen/fiabilidad de los datasets </t>
         </is>
       </c>
     </row>
@@ -670,7 +686,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">El significado de los conceptos/variables/unidades que se manejan están claros desde el principio y se explican claramente en la memoria. </t>
+          <t>xml:space="preserve"&gt;El significado de los conceptos/variables/unidades que se manejan están claros desde el principio y se explican claramente en la memoria. </t>
         </is>
       </c>
     </row>
@@ -682,12 +698,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elección correcta atributos para PCA: al menos cuatro atributos de interés e independientes por área geográfica. Se han fijado/filtrado correctamente las posibles variables libres . </t>
+          <t>xml:space="preserve"&gt;Elección correcta atributos para PCA: al menos cuatro atributos de interés e independientes por área geográfica. Se han fijado/filtrado correctamente las posibles variables libres . </t>
         </is>
       </c>
     </row>
     <row r="20" ht="31.95" customHeight="1">
-      <c r="A20" s="2" t="n"/>
+      <c r="A20" s="2"/>
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Visualizaciones en la memoria</t>
@@ -714,7 +730,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gráficas de calidad profesional: sin textos solapados ni cortados, sin códigos en las etiquetas (salvo grupos edad). Tamaño fuente legible adecuado, autocontenidos (se entienden, sin ambigüedad, con la información que hay en el gráfico), si es necesario, añadir un caption en el chunk para explicar mejor.  Para que un proyecto sea APTO, todos los gráficos deben verificar estos requisitos de calidad. </t>
+          <t>xml:space="preserve"&gt;Gráficas de calidad profesional: sin textos solapados ni cortados, sin códigos en las etiquetas (salvo grupos edad). Tamaño fuente legible adecuado, autocontenidos (se entienden, sin ambigüedad, con la información que hay en el gráfico), si es necesario, añadir un caption en el chunk para explicar mejor.  Para que un proyecto sea APTO, todos los gráficos deben verificar estos requisitos de calidad. </t>
         </is>
       </c>
     </row>
@@ -726,7 +742,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Todas las gráficas dinámicas. </t>
+          <t>xml:space="preserve"&gt;Todas las gráficas dinámicas. </t>
         </is>
       </c>
     </row>
@@ -755,7 +771,7 @@
       </c>
     </row>
     <row r="26" ht="31.95" customHeight="1">
-      <c r="A26" s="2" t="n"/>
+      <c r="A26" s="2"/>
       <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -847,7 +863,7 @@
       </c>
     </row>
     <row r="34" ht="31.95" customHeight="1">
-      <c r="A34" s="2" t="n"/>
+      <c r="A34" s="2"/>
       <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Seguimiento y dedicación</t>
@@ -860,10 +876,8 @@
           <t>1,2,3</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Uso Google Sheet para el control dedicación proyecto</t>
-        </is>
+      <c r="B35" s="7" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -880,5 +894,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Aclara que la entrega se sube sin comprimir (sin .zip)
Republicación desde el curso privado: ver detalle en el commit 0a23514 de
AEDV_2026_2027.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RubricaEvaluaciónProyectoPersonal.xlsx
+++ b/RubricaEvaluaciónProyectoPersonal.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t xml:space="preserve">Preguntas de investigación: se plantean preguntas de investigación interesantes, concretas y que se pueden responder con los datos, que justifican la elección de los datasets y cubren todos los datasets elegidos (no puede haber datasets sin una pregunta que los justifique). La estrategia de selección y el uso de la IA se describen en Comprensión del negocio. Las preguntas iniciales se van refinando por iteraciones a partir del análisis de los datos y se responden en las conclusiones.</t>
   </si>
@@ -22,6 +22,9 @@
   </si>
   <si>
     <t xml:space="preserve">Entrega memoria en html y código en Rmd que solo use librerías usadas en la asignatura, con ficheros de datos en formato RDS. El código debe incluir todo lo necesario para compilar localmente en cualquier ordenador, incluida la imagen de portada como fichero local (no un enlace externo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El nombre de los archivos Rmd y html entregados empieza por el nombre y apellido 1 del alumno. Los ficheros se suben sueltos al Campus Virtual, nunca comprimidos en un .zip o .rar.</t>
   </si>
 </sst>
 </file>
@@ -572,10 +575,8 @@
           <t>1,2,3</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>El nombre de los archivos Rmd y html entregados empieza por el nombre y apellido 1 del alumno</t>
-        </is>
+      <c r="B8" s="7" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="9" ht="31.95" customHeight="1">

</xml_diff>

<commit_message>
Explicita que la memoria se entrega sin código R visible (echo=FALSE)
Republicación desde el curso privado: ver detalle en el commit 6f0d29c de
AEDV_2026_2027.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RubricaEvaluaciónProyectoPersonal.xlsx
+++ b/RubricaEvaluaciónProyectoPersonal.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t xml:space="preserve">Preguntas de investigación: se plantean preguntas de investigación interesantes, concretas y que se pueden responder con los datos, que justifican la elección de los datasets y cubren todos los datasets elegidos (no puede haber datasets sin una pregunta que los justifique). La estrategia de selección y el uso de la IA se describen en Comprensión del negocio. Las preguntas iniciales se van refinando por iteraciones a partir del análisis de los datos y se responden en las conclusiones.</t>
   </si>
@@ -25,6 +25,9 @@
   </si>
   <si>
     <t xml:space="preserve">El nombre de los archivos Rmd y html entregados empieza por el nombre y apellido 1 del alumno. Los ficheros se suben sueltos al Campus Virtual, nunca comprimidos en un .zip o .rar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texto atractivo y fácil de leer, bien formateado, sin rastros de R: ni código visible (echo=FALSE), ni mensajes de carga de librerías ni advertencias, y sin toc: true al principio.</t>
   </si>
 </sst>
 </file>
@@ -593,10 +596,8 @@
           <t>1,2,3</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Texto atractivo y fácil de leer, bien formateado, sin rastros de R (no poner toc: true al principio)</t>
-        </is>
+      <c r="B10" s="5" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="11" ht="31.95" customHeight="1">

</xml_diff>

<commit_message>
Rúbrica: criterio 3 (documento revisado por el alumno), recuadro de indicios de texto de IA sin revisar y errores graves en las gráficas
</commit_message>
<xml_diff>
--- a/RubricaEvaluaciónProyectoPersonal.xlsx
+++ b/RubricaEvaluaciónProyectoPersonal.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t xml:space="preserve">Preguntas de investigación: se plantean preguntas de investigación interesantes, concretas y que se pueden responder con los datos, que justifican la elección de los datasets y cubren todos los datasets elegidos (no puede haber datasets sin una pregunta que los justifique). La estrategia de selección y el uso de la IA se describen en Comprensión del negocio. Las preguntas iniciales se van refinando por iteraciones a partir del análisis de los datos y se responden en las conclusiones.</t>
   </si>
@@ -28,6 +28,105 @@
   </si>
   <si>
     <t xml:space="preserve">Texto atractivo y fácil de leer, bien formateado, sin rastros de R: ni código visible (echo=FALSE), ni mensajes de carga de librerías ni advertencias, y sin toc: true al principio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega y formato t&amp;#233;cnico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,2,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inclusi&amp;#243;n de un enlace al Dashboard del proyecto alojado en el servidor shiny del DIS que funcione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texto y estructura de la memoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texto coherente e ideas y desarrollos interconectados entre s&amp;#237; con un hilo conductor com&amp;#250;n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt; Todas las secciones est&amp;#225;n completadas correctamente siguiendo la metodolog&amp;#237;a CRISP-DM </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las secciones de la memoria se ajustan al modelo y cada cosa va en la secci&amp;#243;n que le corresponde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las aportaciones y conclusiones reflejan bien el trabajo realizado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comprensi&amp;#243;n y preparaci&amp;#243;n de los datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;Incluye correctamente la informaci&amp;#243;n/origen/fiabilidad de los datasets </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se describe en detalle el procesado inicial de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;El significado de los conceptos/variables/unidades que se manejan est&amp;#225;n claros desde el principio y se explican claramente en la memoria. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;Elecci&amp;#243;n correcta atributos para PCA: al menos cuatro atributos de inter&amp;#233;s e independientes por &amp;#225;rea geogr&amp;#225;fica. Se han fijado/filtrado correctamente las posibles variables libres . </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visualizaciones en la memoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las primeras gr&amp;#225;ficas deben ilustrar los conceptos utilizados de forma general y clara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;Gr&amp;#225;ficas de calidad profesional: sin textos solapados ni cortados, sin c&amp;#243;digos en las etiquetas (salvo grupos edad). Tama&amp;#241;o fuente legible adecuado, autocontenidos (se entienden, sin ambig&amp;#252;edad, con la informaci&amp;#243;n que hay en el gr&amp;#225;fico), si es necesario, a&amp;#241;adir un caption en el chunk para explicar mejor.  Para que un proyecto sea APTO, todos los gr&amp;#225;ficos deben verificar estos requisitos de calidad. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;Todas las gr&amp;#225;ficas din&amp;#225;micas. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">En la memoria, no repetir la misma gr&amp;#225;fica m&amp;#250;ltiples veces cambiando los datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gr&amp;#225;ficas de disco, barra, HeatMap y diagramas de caja en la memoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El dashboard est&amp;#225; bien dise&amp;#241;ado e ilustra los datos en su m&amp;#225;xima generalidad. Aparecen y se gestionan todas las variables originales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: contiene series temporales con facet_wrap para exploraci&amp;#243;n profunda de los datos, con la opci&amp;#243;n de dibujar varios atributos en cada gr&amp;#225;fica individual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: contiene modelos ARIMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: contiene mapas coropl&amp;#233;ticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard : contiene comparaci&amp;#243;n de atributos incluyendo Yeo-Johnson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: incluye an&amp;#225;lisis de atributos con matriz de correlaci&amp;#243;n y PCA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todas la variables en el dashboard se deben fijar din&amp;#225;micamente con Inputs. No fijar valores a mano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguimiento y dedicaci&amp;#243;n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El trabajo realizado es coherente con las horas de dedicaci&amp;#243;n al proyecto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento revisado por el alumno: el texto, el código y las gráficas muestran que el alumno ha leído, entendido y corregido todo lo que entrega, también lo generado con ayuda de la IA. Se tienen en cuenta como indicios de un documento no revisado: texto excesivamente largo, retórico o grandilocuente; preguntas de investigación enrevesadas o que los datos no pueden responder; afirmaciones no justificadas por un gráfico o una tabla, en especial las causales basadas solo en una correlación; texto que no coincide con los resultados e interpretaciones genéricas; técnicas de análisis que no se ven en el libro y código que no sigue su estilo; restos de la conversación con la IA; bibliografía que no existe o no se ha consultado; código sobrante (librerías, funciones o chunks que no se usan); comentarios de código excesivos u obvios; y gráficos generados por la IA con errores graves sin revisar. Afecta a la calificación del proyecto y, si el resultado es muy deficiente, la entrega puede calificarse como NO APTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento revisado por el alumno: el texto, el código y las gráficas muestran que el alumno ha leído, entendido y corregido todo lo que entrega, incluido lo generado con la IA. Indicios de lo contrario: texto excesivamente largo o grandilocuente, preguntas de investigación enrevesadas, afirmaciones no justificadas (en especial causales a partir de una correlación), texto que no coincide con los resultados, técnicas o estilo de código que no están en el libro, restos de la conversación con la IA, bibliografía no consultada, código sobrante, comentarios de código excesivos u obvios y gráficos con errores graves sin revisar. Afecta a la calificación y, si el resultado es muy deficiente, la entrega puede ser NO APTA.</t>
   </si>
 </sst>
 </file>
@@ -512,7 +611,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="16.05" customHeight="1">
+    <row r="2" ht="19.95" customHeight="1">
       <c r="A2" s="2"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -520,7 +619,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="31.95" customHeight="1">
+    <row r="3" ht="49" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>1,2,3</t>
@@ -532,7 +631,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="31.95" customHeight="1">
+    <row r="4" ht="94" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>1,2,3</t>
@@ -542,356 +641,256 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="40.2" customHeight="1">
-      <c r="A5" s="2"/>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Entrega y formato técnico</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31.95" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="s">
+    <row r="5" ht="139" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" ht="19.95" customHeight="1">
+      <c r="A6" s="2"/>
+      <c r="B6" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" ht="64" customHeight="1">
+      <c r="A7" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" ht="31.95" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Inclusión de un enlace al Dashboard del proyecto alojado en el servidor shiny del DIS que funcione</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16.05" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="s">
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" ht="49" customHeight="1">
+      <c r="A9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" ht="31.95" customHeight="1">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Texto y estructura de la memoria</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="31.95" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="s">
+    <row r="10" ht="19.95" customHeight="1">
+      <c r="A10" s="2"/>
+      <c r="B10" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" ht="49" customHeight="1">
+      <c r="A11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" ht="31.95" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Texto coherente e ideas y desarrollos interconectados entre sí con un hilo conductor común</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="31.95" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>xml:space="preserve"&gt; Todas las secciones están completadas correctamente siguiendo la metodología CRISP-DM </t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="31.95" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Las secciones de la memoria se ajustan al modelo y cada cosa va en la sección que le corresponde</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16.05" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Las aportaciones y conclusiones reflejan bien el trabajo realizado</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="31.95" customHeight="1">
-      <c r="A15" s="2"/>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Comprensión y preparación de los datos</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="31.95" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>xml:space="preserve"&gt;Incluye correctamente la información/origen/fiabilidad de los datasets </t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="31.95" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>2,3</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Se describe en detalle el procesado inicial de datos</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="31.95" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>xml:space="preserve"&gt;El significado de los conceptos/variables/unidades que se manejan están claros desde el principio y se explican claramente en la memoria. </t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16.05" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>xml:space="preserve"&gt;Elección correcta atributos para PCA: al menos cuatro atributos de interés e independientes por área geográfica. Se han fijado/filtrado correctamente las posibles variables libres . </t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="31.95" customHeight="1">
-      <c r="A20" s="2"/>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Visualizaciones en la memoria</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="63.6" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>2,3</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Las primeras gráficas deben ilustrar los conceptos utilizados de forma general y clara</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="31.95" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>2,3</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>xml:space="preserve"&gt;Gráficas de calidad profesional: sin textos solapados ni cortados, sin códigos en las etiquetas (salvo grupos edad). Tamaño fuente legible adecuado, autocontenidos (se entienden, sin ambigüedad, con la información que hay en el gráfico), si es necesario, añadir un caption en el chunk para explicar mejor.  Para que un proyecto sea APTO, todos los gráficos deben verificar estos requisitos de calidad. </t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="31.95" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>xml:space="preserve"&gt;Todas las gráficas dinámicas. </t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="31.95" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>2,3</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>En la memoria, no repetir la misma gráfica múltiples veces cambiando los datos</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16.05" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>2,3</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Gráficas de disco, barra, HeatMap y diagramas de caja en la memoria</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="31.95" customHeight="1">
-      <c r="A26" s="2"/>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="31.95" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>El dashboard está bien diseñado e ilustra los datos en su máxima generalidad. Aparecen y se gestionan todas las variables originales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="31.95" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Dashboard: contiene series temporales con facet_wrap para exploración profunda de los datos, con la opción de dibujar varios atributos en cada gráfica individual</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="31.95" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Dashboard: contiene modelos ARIMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="31.95" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Dashboard: contiene mapas coropléticos</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="31.95" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Dashboard : contiene comparación de atributos incluyendo Yeo-Johnson</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="31.95" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Dashboard: incluye análisis de atributos con matriz de correlación y PCA</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16.05" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Todas la variables en el dashboard se deben fijar dinámicamente con Inputs. No fijar valores a mano</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="31.95" customHeight="1">
-      <c r="A34" s="2"/>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Seguimiento y dedicación</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="31.95" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="s">
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" ht="19" customHeight="1">
+      <c r="A15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" ht="19.95" customHeight="1">
+      <c r="A16" s="2"/>
+      <c r="B16" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" ht="19" customHeight="1">
+      <c r="A18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" ht="49" customHeight="1">
+      <c r="A20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" ht="19.95" customHeight="1">
+      <c r="A21" s="2"/>
+      <c r="B21" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" ht="94" customHeight="1">
+      <c r="A23" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" ht="19" customHeight="1">
+      <c r="A24" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" ht="19" customHeight="1">
+      <c r="A25" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" ht="19" customHeight="1">
+      <c r="A26" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" ht="19.95" customHeight="1">
+      <c r="A27" s="2"/>
+      <c r="B27" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1">
+      <c r="A29" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1">
+      <c r="A30" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" ht="19" customHeight="1">
+      <c r="A31" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" ht="19" customHeight="1">
+      <c r="A32" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" ht="19" customHeight="1">
+      <c r="A33" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" ht="19.95" customHeight="1">
+      <c r="A35" s="2"/>
+      <c r="B35" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" ht="49" customHeight="1">
+      <c r="A36" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>1,2,3</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>El trabajo realizado es coherente con las horas de dedicación al proyecto.</t>
-        </is>
+    <row r="37" ht="19" customHeight="1">
+      <c r="A37" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
README: callout con los errores a evitar en los gráficos; sin la mención a las afirmaciones causales
</commit_message>
<xml_diff>
--- a/RubricaEvaluaciónProyectoPersonal.xlsx
+++ b/RubricaEvaluaciónProyectoPersonal.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t xml:space="preserve">Preguntas de investigación: se plantean preguntas de investigación interesantes, concretas y que se pueden responder con los datos, que justifican la elección de los datasets y cubren todos los datasets elegidos (no puede haber datasets sin una pregunta que los justifique). La estrategia de selección y el uso de la IA se describen en Comprensión del negocio. Las preguntas iniciales se van refinando por iteraciones a partir del análisis de los datos y se responden en las conclusiones.</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t xml:space="preserve">Documento revisado por el alumno: el texto, el código y las gráficas muestran que el alumno ha leído, entendido y corregido todo lo que entrega, incluido lo generado con la IA. Indicios de lo contrario: texto excesivamente largo o grandilocuente, preguntas de investigación enrevesadas, afirmaciones no justificadas (en especial causales a partir de una correlación), texto que no coincide con los resultados, técnicas o estilo de código que no están en el libro, restos de la conversación con la IA, bibliografía no consultada, código sobrante, comentarios de código excesivos u obvios y gráficos con errores graves sin revisar. Afecta a la calificación y, si el resultado es muy deficiente, la entrega puede ser NO APTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento revisado por el alumno: el texto, el código y las gráficas muestran que el alumno ha leído, entendido y corregido todo lo que entrega, incluido lo generado con la IA. Indicios de lo contrario: texto excesivamente largo o grandilocuente, preguntas de investigación enrevesadas, afirmaciones no justificadas, texto que no coincide con los resultados, técnicas o estilo de código que no están en el libro, restos de la conversación con la IA, bibliografía no consultada, código sobrante, comentarios de código excesivos u obvios y gráficos con errores graves sin revisar. Afecta a la calificación y, si el resultado es muy deficiente, la entrega puede ser NO APTA.</t>
   </si>
 </sst>
 </file>
@@ -641,12 +644,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="139" customHeight="1">
+    <row r="5" ht="124" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" ht="19.95" customHeight="1">

</xml_diff>

<commit_message>
README: indicio de código imposible de entender con lo visto en el libro
</commit_message>
<xml_diff>
--- a/RubricaEvaluaciónProyectoPersonal.xlsx
+++ b/RubricaEvaluaciónProyectoPersonal.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t xml:space="preserve">Preguntas de investigación: se plantean preguntas de investigación interesantes, concretas y que se pueden responder con los datos, que justifican la elección de los datasets y cubren todos los datasets elegidos (no puede haber datasets sin una pregunta que los justifique). La estrategia de selección y el uso de la IA se describen en Comprensión del negocio. Las preguntas iniciales se van refinando por iteraciones a partir del análisis de los datos y se responden en las conclusiones.</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t xml:space="preserve">Documento revisado por el alumno: el texto, el código y las gráficas muestran que el alumno ha leído, entendido y corregido todo lo que entrega, incluido lo generado con la IA. Indicios de lo contrario: texto excesivamente largo o grandilocuente, preguntas de investigación enrevesadas, afirmaciones no justificadas, texto que no coincide con los resultados, técnicas o estilo de código que no están en el libro, restos de la conversación con la IA, bibliografía no consultada, código sobrante, comentarios de código excesivos u obvios y gráficos con errores graves sin revisar. Afecta a la calificación y, si el resultado es muy deficiente, la entrega puede ser NO APTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento revisado por el alumno: el texto, el código y las gráficas muestran que el alumno ha leído, entendido y corregido todo lo que entrega, incluido lo generado con la IA. Indicios de lo contrario: texto excesivamente largo o grandilocuente, preguntas de investigación enrevesadas, afirmaciones no justificadas, texto que no coincide con los resultados, técnicas o estilo de código que no están en el libro, código imposible de entender a partir de los códigos y técnicas del libro, restos de la conversación con la IA, bibliografía no consultada, código sobrante, comentarios de código excesivos u obvios y gráficos con errores graves sin revisar. Afecta a la calificación y, si el resultado es muy deficiente, la entrega puede ser NO APTA.</t>
   </si>
 </sst>
 </file>
@@ -644,12 +647,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="124" customHeight="1">
+    <row r="5" ht="139" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" ht="19.95" customHeight="1">

</xml_diff>

<commit_message>
La imagen de portada puede ser una URL; si es un fichero local hay que entregarla (README, modelo y rúbrica)
</commit_message>
<xml_diff>
--- a/RubricaEvaluaciónProyectoPersonal.xlsx
+++ b/RubricaEvaluaciónProyectoPersonal.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t xml:space="preserve">Preguntas de investigación: se plantean preguntas de investigación interesantes, concretas y que se pueden responder con los datos, que justifican la elección de los datasets y cubren todos los datasets elegidos (no puede haber datasets sin una pregunta que los justifique). La estrategia de selección y el uso de la IA se describen en Comprensión del negocio. Las preguntas iniciales se van refinando por iteraciones a partir del análisis de los datos y se responden en las conclusiones.</t>
   </si>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t xml:space="preserve">Documento revisado por el alumno: el texto, el código y las gráficas muestran que el alumno ha leído, entendido y corregido todo lo que entrega, incluido lo generado con la IA. Indicios de lo contrario: texto excesivamente largo o grandilocuente, preguntas de investigación enrevesadas, afirmaciones no justificadas, texto que no coincide con los resultados, técnicas o estilo de código que no están en el libro, código imposible de entender a partir de los códigos y técnicas del libro, restos de la conversación con la IA, bibliografía no consultada, código sobrante, comentarios de código excesivos u obvios y gráficos con errores graves sin revisar. Afecta a la calificación y, si el resultado es muy deficiente, la entrega puede ser NO APTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega memoria en html y código en Rmd que solo use librerías usadas en la asignatura, con ficheros de datos en formato RDS. El código debe incluir todo lo necesario para compilar localmente en cualquier ordenador, incluida la imagen de portada si es un fichero local.</t>
   </si>
 </sst>
 </file>
@@ -666,7 +669,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">

</xml_diff>

<commit_message>
Sección Dashboard y rúbrica ajustadas a los cuadros de mandos de referencia; tildes de la rúbrica corregidas
</commit_message>
<xml_diff>
--- a/RubricaEvaluaciónProyectoPersonal.xlsx
+++ b/RubricaEvaluaciónProyectoPersonal.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
   <si>
     <t xml:space="preserve">Preguntas de investigación: se plantean preguntas de investigación interesantes, concretas y que se pueden responder con los datos, que justifican la elección de los datasets y cubren todos los datasets elegidos (no puede haber datasets sin una pregunta que los justifique). La estrategia de selección y el uso de la IA se describen en Comprensión del negocio. Las preguntas iniciales se van refinando por iteraciones a partir del análisis de los datos y se responden en las conclusiones.</t>
   </si>
@@ -136,6 +136,96 @@
   </si>
   <si>
     <t xml:space="preserve">Entrega memoria en html y código en Rmd que solo use librerías usadas en la asignatura, con ficheros de datos en formato RDS. El código debe incluir todo lo necesario para compilar localmente en cualquier ordenador, incluida la imagen de portada si es un fichero local.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRITERIOS EVALUACIÓN PROYECTO PERSONAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcance y calidad del trabajo realizado. Este es el factor determinante en la evaluación y puede considerarse como una valoración global que incluye todos los criterios siguientes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega y formato técnico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inclusión de un enlace al Dashboard del proyecto alojado en el servidor shiny del DIS que funcione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texto coherente e ideas y desarrollos interconectados entre sí con un hilo conductor común</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt; Todas las secciones están completadas correctamente siguiendo la metodología CRISP-DM </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las secciones de la memoria se ajustan al modelo y cada cosa va en la sección que le corresponde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comprensión y preparación de los datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;Incluye correctamente la información/origen/fiabilidad de los datasets </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;El significado de los conceptos/variables/unidades que se manejan están claros desde el principio y se explican claramente en la memoria. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;Elección correcta atributos para PCA: al menos cuatro atributos de interés e independientes por área geográfica. Se han fijado/filtrado correctamente las posibles variables libres . </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las primeras gráficas deben ilustrar los conceptos utilizados de forma general y clara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;Gráficas de calidad profesional: sin textos solapados ni cortados, sin códigos en las etiquetas (salvo grupos edad). Tamaño fuente legible adecuado, autocontenidos (se entienden, sin ambigüedad, con la información que hay en el gráfico), si es necesario, añadir un caption en el chunk para explicar mejor.  Para que un proyecto sea APTO, todos los gráficos deben verificar estos requisitos de calidad. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">xml:space="preserve"&gt;Todas las gráficas dinámicas. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">En la memoria, no repetir la misma gráfica múltiples veces cambiando los datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gráficas de disco, barra, HeatMap y diagramas de caja en la memoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El dashboard está bien diseñado e ilustra los datos en su máxima generalidad. Aparecen y se gestionan todas las variables originales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: contiene series temporales con facet_wrap para exploración profunda de los datos, con la opción de dibujar varios atributos en cada gráfica individual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: contiene mapas coropléticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard : contiene comparación de atributos incluyendo Yeo-Johnson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: incluye análisis de atributos con matriz de correlación y PCA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todas la variables en el dashboard se deben fijar dinámicamente con Inputs. No fijar valores a mano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguimiento y dedicación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El trabajo realizado es coherente con las horas de dedicación al proyecto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El dashboard está bien diseñado e ilustra los datos en su máxima generalidad. Aparecen y se gestionan todas las variables originales. Incluye como páginas los cinco cuadros de mandos de referencia de la asignatura adaptados a los datos del proyecto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: contiene series temporales con facet_wrap para exploración profunda de los datos, con la opción de dibujar varios atributos en cada gráfica individual (referencia: Dashboard_exploracion_series.Rmd).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: contiene predicción de series temporales con ARIMA o STL + ARIMA, con el error del ajuste y los tests de ruido blanco de los residuos (referencia: Dashboard_prediccion_series.Rmd).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: contiene mapas coropléticos (referencia: Dashboard_mapa_coropletico.Rmd).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: contiene comparación de dos atributos incluyendo Yeo-Johnson, con el error del ajuste y los tests de los residuos (referencia: Dashboard_atributos_comparacion.Rmd).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard: incluye análisis de atributos con matriz de correlación, PCA y k-means (referencia: Dashboard_atributos_analisis.Rmd).</t>
   </si>
 </sst>
 </file>
@@ -614,10 +704,8 @@
           <t>ENTREGAS</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>CRITERIOS EVALUACIÓN PROYECTO PERSONAL</t>
-        </is>
+      <c r="B1" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="2" ht="19.95" customHeight="1">
@@ -634,10 +722,8 @@
           <t>1,2,3</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Alcance y calidad del trabajo realizado. Este es el factor determinante en la evaluación y puede considerarse como una valoración global que incluye todos los criterios siguientes.</t>
-        </is>
+      <c r="B3" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="4" ht="94" customHeight="1">
@@ -661,7 +747,7 @@
     <row r="6" ht="19.95" customHeight="1">
       <c r="A6" s="2"/>
       <c r="B6" s="3" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" ht="64" customHeight="1">
@@ -677,7 +763,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>8</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" ht="49" customHeight="1">
@@ -707,7 +793,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
@@ -715,7 +801,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
@@ -723,7 +809,7 @@
         <v>6</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1">
@@ -737,7 +823,7 @@
     <row r="16" ht="19.95" customHeight="1">
       <c r="A16" s="2"/>
       <c r="B16" s="3" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" ht="34" customHeight="1">
@@ -745,7 +831,7 @@
         <v>6</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>15</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
@@ -761,7 +847,7 @@
         <v>6</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" ht="49" customHeight="1">
@@ -769,7 +855,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" ht="19.95" customHeight="1">
@@ -783,7 +869,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" ht="94" customHeight="1">
@@ -791,7 +877,7 @@
         <v>16</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
@@ -799,7 +885,7 @@
         <v>7</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" ht="19" customHeight="1">
@@ -807,7 +893,7 @@
         <v>16</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" ht="19" customHeight="1">
@@ -815,7 +901,7 @@
         <v>16</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" ht="19.95" customHeight="1">
@@ -824,28 +910,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" ht="34" customHeight="1">
+    <row r="28" ht="49" customHeight="1">
       <c r="A28" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29" ht="34" customHeight="1">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" ht="49" customHeight="1">
       <c r="A29" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" ht="19" customHeight="1">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" ht="49" customHeight="1">
       <c r="A30" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" ht="19" customHeight="1">
@@ -853,23 +939,23 @@
         <v>7</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" ht="19" customHeight="1">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" ht="34" customHeight="1">
       <c r="A32" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" ht="19" customHeight="1">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1">
       <c r="A33" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>32</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" ht="34" customHeight="1">
@@ -877,13 +963,13 @@
         <v>7</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" ht="19.95" customHeight="1">
       <c r="A35" s="2"/>
       <c r="B35" s="3" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" ht="49" customHeight="1">
@@ -899,7 +985,7 @@
         <v>6</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>